<commit_message>
Export Jira + dashboards du 2026-06-15
</commit_message>
<xml_diff>
--- a/jira_export_2026-06-15.xlsx
+++ b/jira_export_2026-06-15.xlsx
@@ -894,7 +894,7 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>172 €/h</t>
+          <t>171 €/h</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>334.2 h</t>
+          <t>338.0 h</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>35.4%</t>
+          <t>35.8%</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>610.8 h</t>
+          <t>607.0 h</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
         <v>0</v>
       </c>
       <c r="K5" s="10" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="L5" s="10" t="inlineStr">
         <is>
@@ -7206,7 +7206,7 @@
         <v>4</v>
       </c>
       <c r="K64" s="13" t="n">
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="L64" s="13" t="inlineStr">
         <is>
@@ -7225,7 +7225,7 @@
         <v>207</v>
       </c>
       <c r="P64" s="14" t="n">
-        <v>55.2</v>
+        <v>51.75</v>
       </c>
     </row>
     <row r="65">
@@ -9838,7 +9838,7 @@
         <v>8</v>
       </c>
       <c r="K101" s="10" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="L101" s="10" t="inlineStr">
         <is>
@@ -11010,7 +11010,7 @@
         <v>15</v>
       </c>
       <c r="K118" s="13" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="L118" s="13" t="inlineStr">
         <is>
@@ -12276,7 +12276,7 @@
         <v>33</v>
       </c>
       <c r="K137" s="10" t="n">
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="L137" s="10" t="inlineStr">
         <is>
@@ -13147,7 +13147,7 @@
         <v>35066.73</v>
       </c>
       <c r="P151" s="17" t="n">
-        <v>172.34</v>
+        <v>171.07</v>
       </c>
     </row>
   </sheetData>
@@ -14086,7 +14086,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>217</v>
+        <v>218.5</v>
       </c>
     </row>
     <row r="7">
@@ -14096,7 +14096,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>176.25</v>
+        <v>177.75</v>
       </c>
     </row>
     <row r="8">
@@ -14146,7 +14146,7 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>16.5</v>
+        <v>16.75</v>
       </c>
     </row>
     <row r="13">
@@ -14166,7 +14166,7 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>74</v>
+        <v>76.25</v>
       </c>
     </row>
     <row r="15">
@@ -14205,13 +14205,13 @@
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>61.75</v>
+        <v>62.25</v>
       </c>
       <c r="C17" s="10" t="n">
         <v>56</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>5.75</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="18">
@@ -14221,13 +14221,13 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>140</v>
       </c>
       <c r="D18" s="21" t="n">
-        <v>-84</v>
+        <v>-82</v>
       </c>
     </row>
     <row r="19">
@@ -14285,13 +14285,13 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>32</v>
+        <v>32.5</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>119</v>
       </c>
       <c r="D22" s="21" t="n">
-        <v>-87</v>
+        <v>-86.5</v>
       </c>
     </row>
     <row r="23">
@@ -14301,13 +14301,13 @@
         </is>
       </c>
       <c r="B23" s="10" t="n">
-        <v>30.5</v>
+        <v>31.25</v>
       </c>
       <c r="C23" s="10" t="n">
         <v>133</v>
       </c>
       <c r="D23" s="22" t="n">
-        <v>-102.5</v>
+        <v>-101.75</v>
       </c>
     </row>
   </sheetData>
@@ -14410,13 +14410,13 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>148.75</v>
+        <v>150.25</v>
       </c>
       <c r="C5" s="10" t="n">
         <v>467.04</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>31.8</v>
+        <v>32.2</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>35.5</v>
@@ -14428,13 +14428,13 @@
         <v>28.5</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>184.25</v>
+        <v>185.75</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>591.58</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>29.6</v>
+        <v>29.8</v>
       </c>
     </row>
   </sheetData>
@@ -14938,11 +14938,11 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>172.34 €</t>
+          <t>171.07 €</t>
         </is>
       </c>
       <c r="C24" s="10" t="n">
-        <v>203.48</v>
+        <v>204.98</v>
       </c>
     </row>
     <row r="25">
@@ -14953,11 +14953,11 @@
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>64.38 €</t>
+          <t>63.76 €</t>
         </is>
       </c>
       <c r="C25" s="13" t="n">
-        <v>153.3</v>
+        <v>154.8</v>
       </c>
     </row>
     <row r="26">
@@ -15684,7 +15684,7 @@
         <v>-72.59999999999999</v>
       </c>
       <c r="I10" s="29" t="n">
-        <v>172.34</v>
+        <v>171.07</v>
       </c>
       <c r="J10" s="28" t="n">
         <v>122</v>
@@ -15729,7 +15729,7 @@
         </is>
       </c>
       <c r="I12" s="17" t="n">
-        <v>820.29</v>
+        <v>819.02</v>
       </c>
       <c r="J12" s="16" t="inlineStr">
         <is>

</xml_diff>